<commit_message>
Atualiza PDS e corrige abas do dashboard
</commit_message>
<xml_diff>
--- a/PLANILHA_ALMOXARIFADO.xlsx
+++ b/PLANILHA_ALMOXARIFADO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\micro\Desktop\moderno\dashboard-obras\github\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enopsengenharia-my.sharepoint.com/personal/roberto_santiago_integra6a_com/Documents/Área de Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D44E1F7-2EE7-4380-AD78-586A52526D15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="370" documentId="13_ncr:1_{84D8276A-01B3-46C2-A84A-D5DB1468D978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C0B974D-ED2D-460F-A29B-256BE08E7EBA}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="13920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="D'avó" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="73">
   <si>
     <t>Descrição</t>
   </si>
@@ -241,29 +241,39 @@
     <t>201 barras</t>
   </si>
   <si>
-    <t>533 barras</t>
-  </si>
-  <si>
-    <t>5 barras</t>
-  </si>
-  <si>
-    <t>519 barras</t>
+    <r>
+      <t xml:space="preserve">TUBO PEAD ESGOTO D 355 ( </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="14"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ver projetos de obras para este material)</t>
+    </r>
   </si>
   <si>
     <t>158 barras</t>
   </si>
   <si>
-    <t xml:space="preserve">TUBO PEAD ESGOTO D 355 </t>
-  </si>
-  <si>
-    <t>( Ver projetos de obras para este material)</t>
+    <t>490 barras</t>
+  </si>
+  <si>
+    <t>4 barras</t>
+  </si>
+  <si>
+    <t>506 barras</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -296,6 +306,14 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -370,6 +388,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -661,39 +683,39 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="B1:C18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="100.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" customWidth="1"/>
+    <col min="2" max="2" width="100.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
     </row>
-    <row r="3" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="5">
-        <v>46178</v>
+        <v>46185</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
     </row>
-    <row r="5" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>66</v>
       </c>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="4" t="s">
         <v>0</v>
       </c>
@@ -701,7 +723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>2</v>
       </c>
@@ -709,7 +731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>3</v>
       </c>
@@ -717,7 +739,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>4</v>
       </c>
@@ -725,7 +747,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>5</v>
       </c>
@@ -733,7 +755,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>6</v>
       </c>
@@ -741,23 +763,23 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>9</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="14" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C14" s="3">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="15" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>18</v>
       </c>
@@ -765,7 +787,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>12</v>
       </c>
@@ -773,15 +795,15 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>55</v>
       </c>
       <c r="C17" s="3">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="18" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>17</v>
       </c>
@@ -806,40 +828,40 @@
   <sheetPr>
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
-  <dimension ref="B1:P36"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B1:C26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="100.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" customWidth="1"/>
+    <col min="2" max="2" width="100.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
     </row>
-    <row r="3" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="5">
-        <v>46178</v>
+        <v>46185</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
     </row>
-    <row r="5" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="4" t="s">
         <v>0</v>
       </c>
@@ -847,63 +869,63 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="3" t="s">
         <v>58</v>
       </c>
       <c r="C8" s="3">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
         <v>59</v>
       </c>
       <c r="C9" s="3">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C10" s="3">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="3" t="s">
         <v>4</v>
       </c>
       <c r="C11" s="3">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C12" s="3">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="13" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C13" s="3">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="15" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
         <v>7</v>
       </c>
@@ -911,7 +933,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
         <v>8</v>
       </c>
@@ -919,7 +941,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
         <v>9</v>
       </c>
@@ -927,7 +949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
         <v>10</v>
       </c>
@@ -935,7 +957,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="3" t="s">
         <v>11</v>
       </c>
@@ -943,7 +965,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="20" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="3" t="s">
         <v>13</v>
       </c>
@@ -951,7 +973,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="3" t="s">
         <v>19</v>
       </c>
@@ -959,31 +981,31 @@
         <v>845</v>
       </c>
     </row>
-    <row r="22" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="23" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="3" t="s">
         <v>56</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="24" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
         <v>15</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="25" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B25" s="3" t="s">
         <v>16</v>
       </c>
@@ -991,17 +1013,12 @@
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
         <v>63</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>57</v>
-      </c>
-    </row>
-    <row r="36" spans="16:16" x14ac:dyDescent="0.3">
-      <c r="P36" t="s">
-        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1023,39 +1040,39 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="B1:C44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="100.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" customWidth="1"/>
+    <col min="2" max="2" width="100.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
     </row>
-    <row r="3" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="5">
-        <v>46178</v>
+        <v>46185</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
     </row>
-    <row r="5" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>65</v>
       </c>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="4" t="s">
         <v>0</v>
       </c>
@@ -1063,7 +1080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="6" t="s">
         <v>22</v>
       </c>
@@ -1071,15 +1088,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C9" s="3">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="10" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="6" t="s">
         <v>24</v>
       </c>
@@ -1087,15 +1104,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="6" t="s">
         <v>25</v>
       </c>
       <c r="C11" s="3">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="12" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="6" t="s">
         <v>26</v>
       </c>
@@ -1103,7 +1120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="6" t="s">
         <v>27</v>
       </c>
@@ -1111,15 +1128,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="6" t="s">
         <v>53</v>
       </c>
       <c r="C14" s="3">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="6" t="s">
         <v>28</v>
       </c>
@@ -1127,15 +1144,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="6" t="s">
         <v>29</v>
       </c>
       <c r="C16" s="3">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="6" t="s">
         <v>30</v>
       </c>
@@ -1143,31 +1160,31 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="6" t="s">
         <v>31</v>
       </c>
       <c r="C18" s="3">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="19" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="6" t="s">
         <v>32</v>
       </c>
       <c r="C19" s="3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="20" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="6" t="s">
         <v>33</v>
       </c>
       <c r="C20" s="3">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="6" t="s">
         <v>34</v>
       </c>
@@ -1175,7 +1192,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="6" t="s">
         <v>35</v>
       </c>
@@ -1183,7 +1200,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="6" t="s">
         <v>36</v>
       </c>
@@ -1191,7 +1208,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="6" t="s">
         <v>37</v>
       </c>
@@ -1199,15 +1216,15 @@
         <v>71</v>
       </c>
     </row>
-    <row r="25" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="6" t="s">
         <v>38</v>
       </c>
       <c r="C25" s="3">
-        <v>1333</v>
-      </c>
-    </row>
-    <row r="26" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1307</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="6" t="s">
         <v>39</v>
       </c>
@@ -1215,7 +1232,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="27" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="6" t="s">
         <v>40</v>
       </c>
@@ -1223,15 +1240,15 @@
         <v>262</v>
       </c>
     </row>
-    <row r="28" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="6" t="s">
         <v>41</v>
       </c>
       <c r="C28" s="3">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="29" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="6" t="s">
         <v>42</v>
       </c>
@@ -1239,7 +1256,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="6" t="s">
         <v>43</v>
       </c>
@@ -1247,15 +1264,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="31" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="6" t="s">
         <v>44</v>
       </c>
       <c r="C31" s="3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="32" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="6" t="s">
         <v>45</v>
       </c>
@@ -1263,7 +1280,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="33" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="6" t="s">
         <v>46</v>
       </c>
@@ -1271,7 +1288,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="6" t="s">
         <v>47</v>
       </c>
@@ -1279,7 +1296,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="6" t="s">
         <v>48</v>
       </c>
@@ -1287,7 +1304,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="6" t="s">
         <v>49</v>
       </c>
@@ -1295,43 +1312,43 @@
         <v>50</v>
       </c>
     </row>
-    <row r="37" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="6" t="s">
         <v>50</v>
       </c>
       <c r="C37" s="3">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="38" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="6" t="s">
         <v>51</v>
       </c>
       <c r="C38" s="3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
     </row>
-    <row r="40" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
     </row>
-    <row r="41" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
     </row>
-    <row r="42" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
     </row>
-    <row r="43" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="43" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
     </row>
-    <row r="44" spans="2:3" ht="18" x14ac:dyDescent="0.35">
+    <row r="44" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
     </row>

</xml_diff>

<commit_message>
Atualizar PDS almoxarifado e seguranca
</commit_message>
<xml_diff>
--- a/PLANILHA_ALMOXARIFADO.xlsx
+++ b/PLANILHA_ALMOXARIFADO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enopsengenharia-my.sharepoint.com/personal/roberto_santiago_integra6a_com/Documents/Área de Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="415" documentId="13_ncr:1_{84D8276A-01B3-46C2-A84A-D5DB1468D978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E44D8E7-A02D-4779-BE90-75CF89970327}"/>
+  <xr:revisionPtr revIDLastSave="455" documentId="13_ncr:1_{84D8276A-01B3-46C2-A84A-D5DB1468D978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93369CD2-1AEB-43F7-886E-2CBCDA1AFC50}"/>
   <bookViews>
-    <workbookView xWindow="-15480" yWindow="-120" windowWidth="15600" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15480" yWindow="-120" windowWidth="15600" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="D'avó" sheetId="3" r:id="rId1"/>
@@ -214,9 +214,6 @@
     <t>CANTEIRO: Bandeirantes</t>
   </si>
   <si>
-    <t>183 Barras</t>
-  </si>
-  <si>
     <t>TUBO PVC RIG JEI/JERI ESG DN 400 CM 6M</t>
   </si>
   <si>
@@ -229,51 +226,41 @@
     <t>RESPONSÁVEL: João</t>
   </si>
   <si>
-    <t>201 barras</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">TUBO PEAD ESGOTO D 355 ( </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="14"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Ver projetos de obras para este material)</t>
-    </r>
-  </si>
-  <si>
     <t>158 barras</t>
   </si>
   <si>
     <t xml:space="preserve">TUBO PVC RIG JEI/JERI ESG DN 200 CM 6M </t>
   </si>
   <si>
-    <t>487 barras</t>
-  </si>
-  <si>
-    <t>3 Barras</t>
-  </si>
-  <si>
-    <t>391Barras</t>
-  </si>
-  <si>
     <t>266 barras</t>
   </si>
   <si>
-    <t>5 barras</t>
+    <t xml:space="preserve">TUBO PEAD ESGOTO D 355 </t>
+  </si>
+  <si>
+    <t>191 barras</t>
+  </si>
+  <si>
+    <t>133 Barras</t>
+  </si>
+  <si>
+    <t>331Barras</t>
+  </si>
+  <si>
+    <t>33 Barras</t>
+  </si>
+  <si>
+    <t>461 barras</t>
+  </si>
+  <si>
+    <t>4 barras</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -306,14 +293,6 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -389,12 +368,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -719,7 +698,7 @@
     </row>
     <row r="3" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="5">
-        <v>46192</v>
+        <v>46198</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>53</v>
@@ -731,7 +710,7 @@
     </row>
     <row r="5" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -792,7 +771,7 @@
         <v>9</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="14" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -866,7 +845,7 @@
     </row>
     <row r="3" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="5">
-        <v>46192</v>
+        <v>46198</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>58</v>
@@ -878,7 +857,7 @@
     </row>
     <row r="5" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -899,7 +878,7 @@
         <v>56</v>
       </c>
       <c r="C8" s="3">
-        <v>100</v>
+        <v>91</v>
       </c>
     </row>
     <row r="9" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -915,7 +894,7 @@
         <v>3</v>
       </c>
       <c r="C10" s="3">
-        <v>3</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -923,7 +902,7 @@
         <v>4</v>
       </c>
       <c r="C11" s="3">
-        <v>0</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -931,7 +910,7 @@
         <v>5</v>
       </c>
       <c r="C12" s="3">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -939,15 +918,15 @@
         <v>6</v>
       </c>
       <c r="C13" s="3">
-        <v>15</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="15" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -979,7 +958,7 @@
         <v>10</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="2:11" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1003,7 +982,7 @@
         <v>18</v>
       </c>
       <c r="C21" s="3">
-        <v>753</v>
+        <v>646</v>
       </c>
     </row>
     <row r="22" spans="2:11" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1011,7 +990,7 @@
         <v>14</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="2:11" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1019,15 +998,15 @@
         <v>55</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B24" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="10"/>
@@ -1043,13 +1022,13 @@
         <v>15</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="D25" s="7"/>
     </row>
     <row r="26" spans="2:11" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B26" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>72</v>
@@ -1087,7 +1066,7 @@
     </row>
     <row r="3" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="5">
-        <v>46192</v>
+        <v>46198</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>51</v>
@@ -1099,7 +1078,7 @@
     </row>
     <row r="5" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C5" s="3"/>
     </row>
@@ -1128,7 +1107,7 @@
         <v>22</v>
       </c>
       <c r="C9" s="3">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="10" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1144,7 +1123,7 @@
         <v>24</v>
       </c>
       <c r="C11" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1152,7 +1131,7 @@
         <v>25</v>
       </c>
       <c r="C12" s="3">
-        <v>0</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1160,7 +1139,7 @@
         <v>26</v>
       </c>
       <c r="C13" s="3">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1168,7 +1147,7 @@
         <v>52</v>
       </c>
       <c r="C14" s="3">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1176,7 +1155,7 @@
         <v>27</v>
       </c>
       <c r="C15" s="3">
-        <v>28</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1184,7 +1163,7 @@
         <v>28</v>
       </c>
       <c r="C16" s="3">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1200,7 +1179,7 @@
         <v>30</v>
       </c>
       <c r="C18" s="3">
-        <v>375</v>
+        <v>343</v>
       </c>
     </row>
     <row r="19" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1208,7 +1187,7 @@
         <v>31</v>
       </c>
       <c r="C19" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1216,7 +1195,7 @@
         <v>32</v>
       </c>
       <c r="C20" s="3">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1256,7 +1235,7 @@
         <v>37</v>
       </c>
       <c r="C25" s="3">
-        <v>1242</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="26" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1272,7 +1251,7 @@
         <v>39</v>
       </c>
       <c r="C27" s="3">
-        <v>262</v>
+        <v>252</v>
       </c>
     </row>
     <row r="28" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1280,7 +1259,7 @@
         <v>40</v>
       </c>
       <c r="C28" s="3">
-        <v>47</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1304,7 +1283,7 @@
         <v>43</v>
       </c>
       <c r="C31" s="3">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1312,7 +1291,7 @@
         <v>44</v>
       </c>
       <c r="C32" s="3">
-        <v>35</v>
+        <v>21</v>
       </c>
     </row>
     <row r="33" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1352,7 +1331,7 @@
         <v>49</v>
       </c>
       <c r="C37" s="3">
-        <v>689</v>
+        <v>646</v>
       </c>
     </row>
     <row r="38" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1360,7 +1339,7 @@
         <v>50</v>
       </c>
       <c r="C38" s="3">
-        <v>0</v>
+        <v>11</v>
       </c>
     </row>
     <row r="39" spans="2:3" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza PDS 17 julho e almoxarifado
</commit_message>
<xml_diff>
--- a/PLANILHA_ALMOXARIFADO.xlsx
+++ b/PLANILHA_ALMOXARIFADO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enopsengenharia-my.sharepoint.com/personal/roberto_santiago_integra6a_com/Documents/Área de Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="644" documentId="13_ncr:1_{84D8276A-01B3-46C2-A84A-D5DB1468D978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{58392DDB-011F-4152-9EFB-C7263EF75DB5}"/>
+  <xr:revisionPtr revIDLastSave="677" documentId="13_ncr:1_{84D8276A-01B3-46C2-A84A-D5DB1468D978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45283611-C4F8-410D-98AE-B985E73C6FFC}"/>
   <bookViews>
-    <workbookView xWindow="-15480" yWindow="-120" windowWidth="15600" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15480" yWindow="-120" windowWidth="15600" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="D'avó" sheetId="3" r:id="rId1"/>
@@ -802,7 +802,7 @@
     </row>
     <row r="3" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="4">
-        <v>46213</v>
+        <v>46219</v>
       </c>
       <c r="C3" s="15" t="s">
         <v>68</v>
@@ -899,7 +899,7 @@
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3">
-        <v>490</v>
+        <v>460</v>
       </c>
     </row>
     <row r="15" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -926,7 +926,7 @@
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3">
-        <v>205</v>
+        <v>180</v>
       </c>
     </row>
     <row r="18" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -964,7 +964,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="4">
-        <v>46213</v>
+        <v>46219</v>
       </c>
       <c r="B1" s="15" t="s">
         <v>63</v>
@@ -1009,7 +1009,7 @@
         <v>64</v>
       </c>
       <c r="C6" s="7">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1020,7 +1020,7 @@
         <v>64</v>
       </c>
       <c r="C7" s="7">
-        <v>44</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1031,7 +1031,7 @@
         <v>64</v>
       </c>
       <c r="C8" s="7">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1042,7 +1042,7 @@
         <v>64</v>
       </c>
       <c r="C9" s="7">
-        <v>126</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1053,7 +1053,7 @@
         <v>64</v>
       </c>
       <c r="C10" s="7">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1108,7 +1108,7 @@
         <v>65</v>
       </c>
       <c r="C15" s="7">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -1119,7 +1119,7 @@
         <v>65</v>
       </c>
       <c r="C16" s="7">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -1130,7 +1130,7 @@
         <v>65</v>
       </c>
       <c r="C17" s="7">
-        <v>184</v>
+        <v>496</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1141,7 +1141,7 @@
         <v>65</v>
       </c>
       <c r="C18" s="7">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -1152,7 +1152,7 @@
         <v>65</v>
       </c>
       <c r="C19" s="7">
-        <v>360</v>
+        <v>308</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -1174,7 +1174,7 @@
         <v>64</v>
       </c>
       <c r="C21" s="7">
-        <v>554</v>
+        <v>534</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1229,7 +1229,7 @@
         <v>64</v>
       </c>
       <c r="C26" s="7">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -1240,7 +1240,7 @@
         <v>64</v>
       </c>
       <c r="C27" s="7">
-        <v>128</v>
+        <v>116</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -1251,7 +1251,7 @@
         <v>64</v>
       </c>
       <c r="C28" s="8">
-        <v>160</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -1283,7 +1283,7 @@
     </row>
     <row r="3" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="4">
-        <v>46205</v>
+        <v>46219</v>
       </c>
       <c r="C3" s="15" t="s">
         <v>66</v>
@@ -1361,7 +1361,7 @@
         <v>71</v>
       </c>
       <c r="D11" s="3">
-        <v>0</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1372,7 +1372,7 @@
         <v>71</v>
       </c>
       <c r="D12" s="3">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1383,7 +1383,7 @@
         <v>71</v>
       </c>
       <c r="D13" s="3">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1405,7 +1405,7 @@
         <v>71</v>
       </c>
       <c r="D15" s="3">
-        <v>232</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1438,7 +1438,7 @@
         <v>71</v>
       </c>
       <c r="D18" s="3">
-        <v>182</v>
+        <v>143</v>
       </c>
     </row>
     <row r="19" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1493,7 +1493,7 @@
         <v>71</v>
       </c>
       <c r="D23" s="3">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1515,7 +1515,7 @@
         <v>71</v>
       </c>
       <c r="D25" s="3">
-        <v>960</v>
+        <v>885</v>
       </c>
     </row>
     <row r="26" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1526,7 +1526,7 @@
         <v>71</v>
       </c>
       <c r="D26" s="3">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1570,7 +1570,7 @@
         <v>71</v>
       </c>
       <c r="D30" s="3">
-        <v>4</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1614,7 +1614,7 @@
         <v>71</v>
       </c>
       <c r="D34" s="3">
-        <v>48</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Atualiza planilha do almoxarifado
</commit_message>
<xml_diff>
--- a/PLANILHA_ALMOXARIFADO.xlsx
+++ b/PLANILHA_ALMOXARIFADO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://enopsengenharia-my.sharepoint.com/personal/roberto_santiago_integra6a_com/Documents/Área de Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="677" documentId="13_ncr:1_{84D8276A-01B3-46C2-A84A-D5DB1468D978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45283611-C4F8-410D-98AE-B985E73C6FFC}"/>
+  <xr:revisionPtr revIDLastSave="711" documentId="13_ncr:1_{84D8276A-01B3-46C2-A84A-D5DB1468D978}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{60ED1ADF-DD33-45F8-B6AB-9807358F4A80}"/>
   <bookViews>
-    <workbookView xWindow="-15480" yWindow="-120" windowWidth="15600" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15480" yWindow="-120" windowWidth="15600" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="D'avó" sheetId="3" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="76">
   <si>
     <t>Descrição</t>
   </si>
@@ -254,6 +254,15 @@
   </si>
   <si>
     <t xml:space="preserve">BLOCO DE CONCRETO CURVO PI </t>
+  </si>
+  <si>
+    <t>CHAPA ARMICO 2,4 m</t>
+  </si>
+  <si>
+    <t>CHAPA ARMICO 1,8 m</t>
+  </si>
+  <si>
+    <t>TAMPÃO FF TL DN 200</t>
   </si>
 </sst>
 </file>
@@ -323,7 +332,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -420,11 +429,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -440,19 +477,11 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -477,6 +506,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -787,7 +828,7 @@
   <sheetPr>
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="B1:D18"/>
+  <dimension ref="B1:D19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="100.28515625" bestFit="1" customWidth="1"/>
@@ -796,46 +837,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
     </row>
     <row r="3" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="4">
-        <v>46219</v>
-      </c>
-      <c r="C3" s="15" t="s">
+        <v>46226</v>
+      </c>
+      <c r="C3" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="D3" s="16"/>
+      <c r="D3" s="12"/>
     </row>
     <row r="4" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="18"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="14"/>
     </row>
     <row r="5" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="20"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="22"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="8" t="s">
         <v>62</v>
       </c>
     </row>
@@ -895,46 +936,55 @@
     </row>
     <row r="14" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="3" t="s">
-        <v>10</v>
+        <v>73</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3">
-        <v>460</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="3" t="s">
-        <v>14</v>
+        <v>74</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3">
-        <v>7</v>
+        <v>600</v>
       </c>
     </row>
     <row r="16" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="3" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3">
-        <v>180</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="3" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3">
         <v>83</v>
       </c>
     </row>
@@ -954,7 +1004,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44132925-C572-48A3-9D39-75CE91966131}">
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="51" bestFit="1" customWidth="1"/>
@@ -964,294 +1014,305 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="4">
-        <v>46219</v>
-      </c>
-      <c r="B1" s="15" t="s">
+        <v>46226</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="16"/>
+      <c r="C1" s="12"/>
     </row>
     <row r="2" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="18"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
     </row>
     <row r="3" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="20"/>
+      <c r="C3" s="16"/>
     </row>
     <row r="4" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="22"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="18"/>
     </row>
     <row r="5" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="8" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C6" s="7">
-        <v>79</v>
+      <c r="C6" s="21">
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C7" s="7">
-        <v>125</v>
+      <c r="C7" s="21">
+        <v>103</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C8" s="7">
-        <v>19</v>
+      <c r="C8" s="21">
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C9" s="7">
-        <v>122</v>
+      <c r="C9" s="21">
+        <v>120</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="21">
         <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="7">
-        <v>191</v>
+      <c r="C11" s="21">
+        <v>177</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+      <c r="A12" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="21">
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="21">
         <v>234</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="21">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="21">
         <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="21">
         <v>247</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C17" s="7">
-        <v>496</v>
+      <c r="C17" s="21">
+        <v>486</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="21">
         <v>29</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="7">
-        <v>308</v>
+      <c r="C19" s="21">
+        <v>299</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C20" s="7">
+      <c r="C20" s="21">
         <v>250</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="7" t="s">
+      <c r="B21" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C21" s="7">
+      <c r="C21" s="21">
         <v>534</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="7" t="s">
+      <c r="B22" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C22" s="7">
-        <v>30</v>
+      <c r="C22" s="21">
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="7" t="s">
+      <c r="B23" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C23" s="7">
+      <c r="C23" s="21">
         <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B24" s="7" t="s">
+      <c r="B24" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C24" s="7">
+      <c r="C24" s="21">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="C25" s="7">
+      <c r="C25" s="21">
         <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="7">
-        <v>36</v>
+      <c r="C26" s="21">
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C27" s="7">
-        <v>116</v>
+      <c r="C27" s="21">
+        <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="8" t="s">
+      <c r="A28" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="8">
-        <v>140</v>
+      <c r="C28" s="21">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" s="21">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1277,51 +1338,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
     </row>
     <row r="3" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="4">
-        <v>46219</v>
-      </c>
-      <c r="C3" s="15" t="s">
+        <v>46226</v>
+      </c>
+      <c r="C3" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="16"/>
+      <c r="D3" s="12"/>
     </row>
     <row r="4" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="3"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="18"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="14"/>
     </row>
     <row r="5" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="20"/>
+      <c r="D5" s="16"/>
     </row>
     <row r="6" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="22"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="18"/>
     </row>
     <row r="7" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="8" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="8" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="9" t="s">
         <v>15</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -1332,18 +1393,18 @@
       </c>
     </row>
     <row r="9" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="9" t="s">
         <v>16</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D9" s="3">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="10" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="9" t="s">
         <v>17</v>
       </c>
       <c r="C10" s="5" t="s">
@@ -1354,29 +1415,29 @@
       </c>
     </row>
     <row r="11" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="9" t="s">
         <v>18</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D11" s="3">
-        <v>42</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="9" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D12" s="3">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="9" t="s">
         <v>20</v>
       </c>
       <c r="C13" s="5" t="s">
@@ -1387,29 +1448,29 @@
       </c>
     </row>
     <row r="14" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="9" t="s">
         <v>44</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D14" s="3">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="9" t="s">
         <v>21</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D15" s="3">
-        <v>116</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="9" t="s">
         <v>22</v>
       </c>
       <c r="C16" s="5" t="s">
@@ -1420,29 +1481,29 @@
       </c>
     </row>
     <row r="17" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="9" t="s">
         <v>23</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D17" s="3">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="9" t="s">
         <v>24</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D18" s="3">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="19" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="9" t="s">
         <v>25</v>
       </c>
       <c r="C19" s="5" t="s">
@@ -1453,18 +1514,18 @@
       </c>
     </row>
     <row r="20" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="9" t="s">
         <v>26</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D20" s="3">
-        <v>34</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="9" t="s">
         <v>27</v>
       </c>
       <c r="C21" s="5" t="s">
@@ -1475,7 +1536,7 @@
       </c>
     </row>
     <row r="22" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="9" t="s">
         <v>28</v>
       </c>
       <c r="C22" s="5" t="s">
@@ -1486,18 +1547,18 @@
       </c>
     </row>
     <row r="23" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="9" t="s">
         <v>29</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D23" s="3">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="9" t="s">
         <v>30</v>
       </c>
       <c r="C24" s="5" t="s">
@@ -1508,29 +1569,29 @@
       </c>
     </row>
     <row r="25" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="9" t="s">
         <v>31</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D25" s="3">
-        <v>885</v>
+        <v>825</v>
       </c>
     </row>
     <row r="26" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="9" t="s">
         <v>32</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D26" s="3">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="9" t="s">
         <v>33</v>
       </c>
       <c r="C27" s="5" t="s">
@@ -1541,7 +1602,7 @@
       </c>
     </row>
     <row r="28" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="9" t="s">
         <v>34</v>
       </c>
       <c r="C28" s="5" t="s">
@@ -1552,7 +1613,7 @@
       </c>
     </row>
     <row r="29" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="9" t="s">
         <v>35</v>
       </c>
       <c r="C29" s="5" t="s">
@@ -1563,7 +1624,7 @@
       </c>
     </row>
     <row r="30" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="9" t="s">
         <v>36</v>
       </c>
       <c r="C30" s="5" t="s">
@@ -1574,7 +1635,7 @@
       </c>
     </row>
     <row r="31" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="9" t="s">
         <v>37</v>
       </c>
       <c r="C31" s="5" t="s">
@@ -1585,7 +1646,7 @@
       </c>
     </row>
     <row r="32" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="9" t="s">
         <v>38</v>
       </c>
       <c r="C32" s="5" t="s">
@@ -1596,7 +1657,7 @@
       </c>
     </row>
     <row r="33" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="11" t="s">
+      <c r="B33" s="9" t="s">
         <v>39</v>
       </c>
       <c r="C33" s="5" t="s">
@@ -1607,7 +1668,7 @@
       </c>
     </row>
     <row r="34" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="9" t="s">
         <v>40</v>
       </c>
       <c r="C34" s="5" t="s">
@@ -1618,7 +1679,7 @@
       </c>
     </row>
     <row r="35" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="11" t="s">
+      <c r="B35" s="9" t="s">
         <v>41</v>
       </c>
       <c r="C35" s="5" t="s">
@@ -1629,18 +1690,18 @@
       </c>
     </row>
     <row r="36" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="9" t="s">
         <v>42</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D36" s="3">
-        <v>473</v>
+        <v>338</v>
       </c>
     </row>
     <row r="37" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="11" t="s">
+      <c r="B37" s="9" t="s">
         <v>43</v>
       </c>
       <c r="C37" s="5" t="s">
@@ -1651,7 +1712,7 @@
       </c>
     </row>
     <row r="38" spans="2:4" s="2" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="9" t="s">
         <v>70</v>
       </c>
       <c r="C38" s="5" t="s">

</xml_diff>